<commit_message>
Popravljanje datoteke Opravljeno delo
</commit_message>
<xml_diff>
--- a/GrilUrska/opravljenoDelo/GrilUrska.xlsx
+++ b/GrilUrska/opravljenoDelo/GrilUrska.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\urska\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\urska\AlmaMaterGIT\alma2026racunalnistvoOblak\GrilUrska\opravljenoDelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E08BFAC-4B08-462D-AA00-5E28AC574AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A93C06F5-C7AC-4C22-A3CF-6D9804BBA302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -690,9 +690,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -718,6 +715,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1536,40 +1536,40 @@
     <row r="3" spans="2:16" ht="201.6" x14ac:dyDescent="0.3">
       <c r="B3" s="11"/>
       <c r="C3" s="12"/>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="P3" s="19" t="s">
+      <c r="P3" s="18" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1580,10 +1580,10 @@
       <c r="C4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>47</v>
       </c>
       <c r="F4" s="4"/>
@@ -1595,7 +1595,7 @@
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
-      <c r="P4" s="20" t="s">
+      <c r="P4" s="19" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1631,30 +1631,30 @@
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="15"/>
-      <c r="P5" s="21" t="s">
+      <c r="P5" s="20" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="144" x14ac:dyDescent="0.3">
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="21" t="s">
         <v>58</v>
       </c>
       <c r="E6" s="4"/>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="22" t="s">
         <v>62</v>
       </c>
       <c r="K6" s="4"/>
@@ -1669,16 +1669,16 @@
       <c r="C7" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="22" t="s">
         <v>59</v>
       </c>
       <c r="H7" s="4"/>
@@ -1692,15 +1692,15 @@
     <row r="8" spans="2:16" ht="244.8" x14ac:dyDescent="0.3">
       <c r="B8" s="9"/>
       <c r="C8" s="10"/>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="22" t="s">
         <v>66</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="22" t="s">
         <v>68</v>
       </c>
       <c r="I8" s="4"/>
@@ -1744,22 +1744,22 @@
     <row r="10" spans="2:16" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B10" s="9"/>
       <c r="C10" s="10"/>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="22" t="s">
         <v>75</v>
       </c>
       <c r="J10" s="4"/>
@@ -1794,10 +1794,10 @@
     <row r="12" spans="2:16" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B12" s="9"/>
       <c r="C12" s="10"/>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="22" t="s">
         <v>77</v>
       </c>
       <c r="F12" s="4"/>
@@ -1817,16 +1817,16 @@
       <c r="C13" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="22" t="s">
         <v>30</v>
       </c>
       <c r="H13" s="4"/>
@@ -1840,12 +1840,12 @@
     <row r="14" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B14" s="9"/>
       <c r="C14" s="10"/>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23" t="s">
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22" t="s">
         <v>79</v>
       </c>
       <c r="H14" s="4"/>
@@ -1886,16 +1886,16 @@
     <row r="16" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B16" s="9"/>
       <c r="C16" s="10"/>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="22" t="s">
         <v>84</v>
       </c>
       <c r="H16" s="4"/>
@@ -1913,10 +1913,10 @@
       <c r="C17" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="22" t="s">
         <v>78</v>
       </c>
       <c r="F17" s="4"/>
@@ -1976,13 +1976,13 @@
     <row r="20" spans="2:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B20" s="9"/>
       <c r="C20" s="10"/>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="22" t="s">
         <v>89</v>
       </c>
       <c r="G20" s="4"/>
@@ -2020,7 +2020,7 @@
     <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B22" s="9"/>
       <c r="C22" s="10"/>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="23" t="s">
         <v>94</v>
       </c>
       <c r="E22" s="4"/>
@@ -2041,19 +2041,19 @@
       <c r="C23" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="G23" s="23" t="s">
+      <c r="G23" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="22" t="s">
         <v>96</v>
       </c>
       <c r="I23" s="4"/>
@@ -2070,7 +2070,7 @@
       <c r="C24" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="23" t="s">
         <v>40</v>
       </c>
       <c r="E24" s="4"/>
@@ -2091,7 +2091,7 @@
       <c r="C25" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D25" s="24" t="s">
+      <c r="D25" s="23" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="4"/>
@@ -2106,13 +2106,13 @@
       <c r="N25" s="15"/>
     </row>
     <row r="26" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="17">
+      <c r="B26" s="16">
         <v>9</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="16" t="s">
+      <c r="C26" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="25" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>